<commit_message>
Add new EDC product and validate AI results
</commit_message>
<xml_diff>
--- a/goods(4).xlsx
+++ b/goods(4).xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="115">
   <si>
     <t>Bags</t>
   </si>
@@ -348,6 +348,18 @@
   </si>
   <si>
     <t>USD</t>
+  </si>
+  <si>
+    <t>Handmade Leather EDC Belt Pouch / Multitool &amp; Folding Knife Sheath / EveryDay Carry Belt Organizer by Alex Polak</t>
+  </si>
+  <si>
+    <t>https://www.etsy.com/listing/4505762718</t>
+  </si>
+  <si>
+    <t>images/edc/4505762718.jpg</t>
+  </si>
+  <si>
+    <t>Handmade black leather EDC pouch displayed with keys, cards and everyday carry accessories</t>
   </si>
 </sst>
 </file>
@@ -736,7 +748,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J19"/>
+  <dimension ref="A1:J20"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -1354,6 +1366,38 @@
         <v>69</v>
       </c>
       <c r="J19" s="8" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="A20" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="C20" t="s">
+        <v>87</v>
+      </c>
+      <c r="D20" t="s">
+        <v>112</v>
+      </c>
+      <c r="E20" t="s">
+        <v>113</v>
+      </c>
+      <c r="F20" t="s">
+        <v>114</v>
+      </c>
+      <c r="G20" t="s">
+        <v>43</v>
+      </c>
+      <c r="H20" t="s">
+        <v>44</v>
+      </c>
+      <c r="I20" s="10">
+        <v>69</v>
+      </c>
+      <c r="J20" s="8" t="s">
         <v>110</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add 3 items to site
</commit_message>
<xml_diff>
--- a/goods(4).xlsx
+++ b/goods(4).xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="124">
   <si>
     <t>Bags</t>
   </si>
@@ -360,6 +360,33 @@
   </si>
   <si>
     <t>Handmade black leather EDC pouch displayed with keys, cards and everyday carry accessories</t>
+  </si>
+  <si>
+    <t>images/edc/4384063617.jpg</t>
+  </si>
+  <si>
+    <t>Handmade Leather EDC Belt Pouch, Minimalist Leather Organizer for Men, Knife &amp; Lighter Holder, Bushcraft Gear, Gift for Him</t>
+  </si>
+  <si>
+    <t>https://www.etsy.com/listing/4384063617</t>
+  </si>
+  <si>
+    <t>Leather Belt Pouch Wallet, Leather Belt Bag, EDC Belt Pocket Organizer with YKK Zipper, Handmade Card and Key Holder, Gift for him</t>
+  </si>
+  <si>
+    <t>https://www.etsy.com/listing/4559330701</t>
+  </si>
+  <si>
+    <t>images/edc/4559330701.jpg</t>
+  </si>
+  <si>
+    <t>Handmade  leather EDC pouch displayed with keys, cards and everyday carry accessories</t>
+  </si>
+  <si>
+    <t>https://www.etsy.com/listing/4524136544</t>
+  </si>
+  <si>
+    <t>images/edc/4524136544.jpg</t>
   </si>
 </sst>
 </file>
@@ -748,13 +775,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J20"/>
+  <dimension ref="A1:J23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="3" width="47.5703125" customWidth="1"/>
     <col min="4" max="4" width="49.85546875" customWidth="1"/>
-    <col min="5" max="6" width="28.85546875" customWidth="1"/>
+    <col min="5" max="5" width="28.85546875" customWidth="1"/>
+    <col min="6" max="6" width="25.140625" customWidth="1"/>
     <col min="7" max="7" width="10.42578125" customWidth="1"/>
     <col min="8" max="8" width="11.42578125" customWidth="1"/>
     <col min="9" max="9" width="9.140625" style="10"/>
@@ -1401,13 +1429,110 @@
         <v>110</v>
       </c>
     </row>
+    <row r="21" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="C21" t="s">
+        <v>84</v>
+      </c>
+      <c r="D21" t="s">
+        <v>117</v>
+      </c>
+      <c r="E21" t="s">
+        <v>115</v>
+      </c>
+      <c r="F21" t="s">
+        <v>106</v>
+      </c>
+      <c r="G21" t="s">
+        <v>43</v>
+      </c>
+      <c r="H21" t="s">
+        <v>44</v>
+      </c>
+      <c r="I21" s="10">
+        <v>69</v>
+      </c>
+      <c r="J21" s="8" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="A22" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="C22" t="s">
+        <v>87</v>
+      </c>
+      <c r="D22" t="s">
+        <v>119</v>
+      </c>
+      <c r="E22" t="s">
+        <v>120</v>
+      </c>
+      <c r="F22" t="s">
+        <v>121</v>
+      </c>
+      <c r="G22" t="s">
+        <v>43</v>
+      </c>
+      <c r="H22" t="s">
+        <v>44</v>
+      </c>
+      <c r="I22" s="10">
+        <v>55</v>
+      </c>
+      <c r="J22" s="8" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="A23" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="C23" t="s">
+        <v>86</v>
+      </c>
+      <c r="D23" t="s">
+        <v>122</v>
+      </c>
+      <c r="E23" t="s">
+        <v>123</v>
+      </c>
+      <c r="F23" t="s">
+        <v>114</v>
+      </c>
+      <c r="G23" t="s">
+        <v>43</v>
+      </c>
+      <c r="H23" t="s">
+        <v>44</v>
+      </c>
+      <c r="I23" s="10">
+        <v>55</v>
+      </c>
+      <c r="J23" s="8" t="s">
+        <v>110</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="D2" r:id="rId1"/>
     <hyperlink ref="D9" r:id="rId2"/>
+    <hyperlink ref="D20" r:id="rId3"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId4"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Add two leather belt pouch product pages
</commit_message>
<xml_diff>
--- a/goods(4).xlsx
+++ b/goods(4).xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="130">
   <si>
     <t>Bags</t>
   </si>
@@ -387,6 +387,24 @@
   </si>
   <si>
     <t>images/edc/4524136544.jpg</t>
+  </si>
+  <si>
+    <t>Handmade Leather Belt Pouch, EDC Waist Bag, Coin Card Holder</t>
+  </si>
+  <si>
+    <t>https://www.etsy.com/listing/1815374701</t>
+  </si>
+  <si>
+    <t>images/edc/1815374701.jpg</t>
+  </si>
+  <si>
+    <t>Brown Leather Belt Pouch, Brown Leather Belt Bag, EDC Pocket Organizer, Compact Belt Holster for Men, gift for him</t>
+  </si>
+  <si>
+    <t>https://www.etsy.com/listing/4590678904</t>
+  </si>
+  <si>
+    <t>images/edc/4590678904.jpg</t>
   </si>
 </sst>
 </file>
@@ -775,7 +793,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J23"/>
+  <dimension ref="A1:J25"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -1385,7 +1403,7 @@
         <v>106</v>
       </c>
       <c r="G19" t="s">
-        <v>43</v>
+        <v>107</v>
       </c>
       <c r="H19" t="s">
         <v>44</v>
@@ -1522,6 +1540,70 @@
         <v>55</v>
       </c>
       <c r="J23" s="8" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A24" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="C24" t="s">
+        <v>86</v>
+      </c>
+      <c r="D24" t="s">
+        <v>125</v>
+      </c>
+      <c r="E24" t="s">
+        <v>126</v>
+      </c>
+      <c r="F24" t="s">
+        <v>121</v>
+      </c>
+      <c r="G24" t="s">
+        <v>43</v>
+      </c>
+      <c r="H24" t="s">
+        <v>44</v>
+      </c>
+      <c r="I24" s="10">
+        <v>69</v>
+      </c>
+      <c r="J24" s="8" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="A25" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="C25" t="s">
+        <v>86</v>
+      </c>
+      <c r="D25" s="6" t="s">
+        <v>128</v>
+      </c>
+      <c r="E25" t="s">
+        <v>129</v>
+      </c>
+      <c r="F25" t="s">
+        <v>121</v>
+      </c>
+      <c r="G25" t="s">
+        <v>43</v>
+      </c>
+      <c r="H25" t="s">
+        <v>44</v>
+      </c>
+      <c r="I25" s="10">
+        <v>69</v>
+      </c>
+      <c r="J25" s="8" t="s">
         <v>110</v>
       </c>
     </row>
@@ -1530,9 +1612,10 @@
     <hyperlink ref="D2" r:id="rId1"/>
     <hyperlink ref="D9" r:id="rId2"/>
     <hyperlink ref="D20" r:id="rId3"/>
+    <hyperlink ref="D25" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId4"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId5"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Add five leather goods product pages
</commit_message>
<xml_diff>
--- a/goods(4).xlsx
+++ b/goods(4).xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="279" uniqueCount="148">
   <si>
     <t>Bags</t>
   </si>
@@ -405,6 +405,60 @@
   </si>
   <si>
     <t>images/edc/4590678904.jpg</t>
+  </si>
+  <si>
+    <t>Handmade Croc Embossed Leather Tote Bag – Structured Luxury Handbag for Everyday</t>
+  </si>
+  <si>
+    <t>Elegant handmade leather tote bag in deep burgundy crocodile embossed leather.</t>
+  </si>
+  <si>
+    <t>https://www.etsy.com/listing/4443159878</t>
+  </si>
+  <si>
+    <t>images/bags/4443159878.jpg</t>
+  </si>
+  <si>
+    <t>Handmade Croc Embossed Leather Tote Bag</t>
+  </si>
+  <si>
+    <t>Horizontal Leather Belt Pouch, Low Profile EDC Card Holder, Stealth Belt Wallet, Gift for him, Alex Polak</t>
+  </si>
+  <si>
+    <t>https://www.etsy.com/listing/4497871197</t>
+  </si>
+  <si>
+    <t>images/edc/4497871197.jpg</t>
+  </si>
+  <si>
+    <t>Horizontal Leather Belt Pouch</t>
+  </si>
+  <si>
+    <t>https://www.etsy.com/listing/4546239570</t>
+  </si>
+  <si>
+    <t>images/edc/4546239570.jpg</t>
+  </si>
+  <si>
+    <t>Handmade Brown Leather Belt Pouch, EDC Carry-All</t>
+  </si>
+  <si>
+    <t>https://www.etsy.com/listing/4361026591</t>
+  </si>
+  <si>
+    <t>images/edc/4361026591.jpg</t>
+  </si>
+  <si>
+    <t>Handmade Brown Leather Belt Pouch</t>
+  </si>
+  <si>
+    <t>https://www.etsy.com/listing/1126874991</t>
+  </si>
+  <si>
+    <t>images/edc/1126874991.jpg</t>
+  </si>
+  <si>
+    <t>Leather EDC Belt Pouch, Coin, Card Holder</t>
   </si>
 </sst>
 </file>
@@ -793,7 +847,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J25"/>
+  <dimension ref="A1:J30"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -1595,7 +1649,7 @@
         <v>121</v>
       </c>
       <c r="G25" t="s">
-        <v>43</v>
+        <v>107</v>
       </c>
       <c r="H25" t="s">
         <v>44</v>
@@ -1604,6 +1658,166 @@
         <v>69</v>
       </c>
       <c r="J25" s="8" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="A26" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="C26" t="s">
+        <v>131</v>
+      </c>
+      <c r="D26" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="E26" t="s">
+        <v>133</v>
+      </c>
+      <c r="F26" t="s">
+        <v>134</v>
+      </c>
+      <c r="G26" t="s">
+        <v>43</v>
+      </c>
+      <c r="H26" t="s">
+        <v>44</v>
+      </c>
+      <c r="I26" s="10">
+        <v>87</v>
+      </c>
+      <c r="J26" s="8" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="A27" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="C27" t="s">
+        <v>86</v>
+      </c>
+      <c r="D27" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="E27" t="s">
+        <v>137</v>
+      </c>
+      <c r="F27" t="s">
+        <v>138</v>
+      </c>
+      <c r="G27" t="s">
+        <v>43</v>
+      </c>
+      <c r="H27" t="s">
+        <v>44</v>
+      </c>
+      <c r="I27" s="10">
+        <v>59</v>
+      </c>
+      <c r="J27" s="8" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="A28" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="C28" t="s">
+        <v>86</v>
+      </c>
+      <c r="D28" s="6" t="s">
+        <v>139</v>
+      </c>
+      <c r="E28" t="s">
+        <v>140</v>
+      </c>
+      <c r="F28" t="s">
+        <v>138</v>
+      </c>
+      <c r="G28" t="s">
+        <v>43</v>
+      </c>
+      <c r="H28" t="s">
+        <v>44</v>
+      </c>
+      <c r="I28" s="10">
+        <v>59</v>
+      </c>
+      <c r="J28" s="8" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A29" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="C29" t="s">
+        <v>86</v>
+      </c>
+      <c r="D29" s="6" t="s">
+        <v>142</v>
+      </c>
+      <c r="E29" t="s">
+        <v>143</v>
+      </c>
+      <c r="F29" t="s">
+        <v>144</v>
+      </c>
+      <c r="G29" t="s">
+        <v>43</v>
+      </c>
+      <c r="H29" t="s">
+        <v>44</v>
+      </c>
+      <c r="I29" s="10">
+        <v>59</v>
+      </c>
+      <c r="J29" s="8" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A30" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C30" t="s">
+        <v>84</v>
+      </c>
+      <c r="D30" s="6" t="s">
+        <v>145</v>
+      </c>
+      <c r="E30" t="s">
+        <v>146</v>
+      </c>
+      <c r="F30" t="s">
+        <v>147</v>
+      </c>
+      <c r="G30" t="s">
+        <v>43</v>
+      </c>
+      <c r="H30" t="s">
+        <v>44</v>
+      </c>
+      <c r="I30" s="10">
+        <v>67</v>
+      </c>
+      <c r="J30" s="8" t="s">
         <v>110</v>
       </c>
     </row>
@@ -1613,9 +1827,14 @@
     <hyperlink ref="D9" r:id="rId2"/>
     <hyperlink ref="D20" r:id="rId3"/>
     <hyperlink ref="D25" r:id="rId4"/>
+    <hyperlink ref="D26" r:id="rId5"/>
+    <hyperlink ref="D27" r:id="rId6"/>
+    <hyperlink ref="D28" r:id="rId7"/>
+    <hyperlink ref="D29" r:id="rId8"/>
+    <hyperlink ref="D30" r:id="rId9"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId5"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId10"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Add Buy now cart and Western Bid checkout
</commit_message>
<xml_diff>
--- a/goods(4).xlsx
+++ b/goods(4).xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="279" uniqueCount="148">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="280" uniqueCount="149">
   <si>
     <t>Bags</t>
   </si>
@@ -459,6 +459,9 @@
   </si>
   <si>
     <t>Leather EDC Belt Pouch, Coin, Card Holder</t>
+  </si>
+  <si>
+    <t>Shipping</t>
   </si>
 </sst>
 </file>
@@ -847,7 +850,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J30"/>
+  <dimension ref="A1:K30"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -861,7 +864,7 @@
     <col min="10" max="10" width="9.140625" style="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>38</v>
       </c>
@@ -892,8 +895,11 @@
       <c r="J1" s="7" t="s">
         <v>109</v>
       </c>
-    </row>
-    <row r="2" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="K1" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -924,8 +930,11 @@
       <c r="J2" s="8" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="3" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="K2">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
@@ -956,8 +965,11 @@
       <c r="J3" s="8" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="4" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="K3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>0</v>
       </c>
@@ -988,8 +1000,11 @@
       <c r="J4" s="8" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="5" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="K4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>0</v>
       </c>
@@ -1020,8 +1035,11 @@
       <c r="J5" s="8" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="6" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="K5">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>1</v>
       </c>
@@ -1052,8 +1070,11 @@
       <c r="J6" s="8" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="7" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="K6">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>1</v>
       </c>
@@ -1084,8 +1105,11 @@
       <c r="J7" s="8" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="8" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="K7">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>2</v>
       </c>
@@ -1116,8 +1140,11 @@
       <c r="J8" s="8" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="9" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="K8">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>2</v>
       </c>
@@ -1148,8 +1175,11 @@
       <c r="J9" s="8" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="10" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="K9">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>2</v>
       </c>
@@ -1180,8 +1210,11 @@
       <c r="J10" s="8" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="11" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="K10">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>2</v>
       </c>
@@ -1212,8 +1245,11 @@
       <c r="J11" s="8" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="12" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="K11">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>2</v>
       </c>
@@ -1244,8 +1280,11 @@
       <c r="J12" s="8" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="13" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="K12">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>2</v>
       </c>
@@ -1276,8 +1315,11 @@
       <c r="J13" s="8" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="14" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="K13">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>3</v>
       </c>
@@ -1308,8 +1350,11 @@
       <c r="J14" s="8" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="15" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="K14">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>3</v>
       </c>
@@ -1340,8 +1385,11 @@
       <c r="J15" s="8" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="16" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="K15">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>3</v>
       </c>
@@ -1372,8 +1420,11 @@
       <c r="J16" s="8" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="17" spans="1:10" ht="60" x14ac:dyDescent="0.25">
+      <c r="K16">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>3</v>
       </c>
@@ -1404,8 +1455,11 @@
       <c r="J17" s="8" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="18" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="K17">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>3</v>
       </c>
@@ -1436,8 +1490,11 @@
       <c r="J18" s="8" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="19" spans="1:10" ht="60" x14ac:dyDescent="0.25">
+      <c r="K18">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" ht="60" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>3</v>
       </c>
@@ -1468,8 +1525,11 @@
       <c r="J19" s="8" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="20" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="K19">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>3</v>
       </c>
@@ -1500,8 +1560,11 @@
       <c r="J20" s="8" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="21" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="K20">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>3</v>
       </c>
@@ -1532,8 +1595,11 @@
       <c r="J21" s="8" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="22" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="K21">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>3</v>
       </c>
@@ -1564,8 +1630,11 @@
       <c r="J22" s="8" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="23" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="K22">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>3</v>
       </c>
@@ -1596,8 +1665,11 @@
       <c r="J23" s="8" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="24" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="K23">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>3</v>
       </c>
@@ -1628,8 +1700,11 @@
       <c r="J24" s="8" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="25" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="K24">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>3</v>
       </c>
@@ -1660,8 +1735,11 @@
       <c r="J25" s="8" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="26" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="K25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>0</v>
       </c>
@@ -1692,8 +1770,11 @@
       <c r="J26" s="8" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="27" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="K26">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>3</v>
       </c>
@@ -1724,8 +1805,11 @@
       <c r="J27" s="8" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="28" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="K27">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" ht="45" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>3</v>
       </c>
@@ -1756,8 +1840,11 @@
       <c r="J28" s="8" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="29" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="K28">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>3</v>
       </c>
@@ -1789,7 +1876,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="30" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>3</v>
       </c>
@@ -1819,6 +1906,9 @@
       </c>
       <c r="J30" s="8" t="s">
         <v>110</v>
+      </c>
+      <c r="K30">
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add product image galleries
</commit_message>
<xml_diff>
--- a/goods(4).xlsx
+++ b/goods(4).xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="283" uniqueCount="152">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="361" uniqueCount="230">
   <si>
     <t>Bags</t>
   </si>
@@ -471,13 +471,247 @@
   </si>
   <si>
     <t>Max Qty</t>
+  </si>
+  <si>
+    <t>Image 2</t>
+  </si>
+  <si>
+    <t>Image 3</t>
+  </si>
+  <si>
+    <t>Image 4</t>
+  </si>
+  <si>
+    <t>images/bags/1894993167_2.jpg</t>
+  </si>
+  <si>
+    <t>images/bags/1894993167_3.jpg</t>
+  </si>
+  <si>
+    <t>images/bags/1894993167_4.jpg</t>
+  </si>
+  <si>
+    <t>images/bags/4346158727_2.jpg</t>
+  </si>
+  <si>
+    <t>images/bags/4346158727_3.jpg</t>
+  </si>
+  <si>
+    <t>images/bags/4346158727_4.jpg</t>
+  </si>
+  <si>
+    <t>images/bags/1827745902_2.jpg</t>
+  </si>
+  <si>
+    <t>images/bags/1827745902_3.jpg</t>
+  </si>
+  <si>
+    <t>images/bags/1827745902_4.jpg</t>
+  </si>
+  <si>
+    <t>images/bags/1774631035_2.jpg</t>
+  </si>
+  <si>
+    <t>images/bags/1774631035_3.jpg</t>
+  </si>
+  <si>
+    <t>images/bags/1774631035_4.jpg</t>
+  </si>
+  <si>
+    <t>images/wallets/1641259664_2.jpg</t>
+  </si>
+  <si>
+    <t>images/wallets/1641259664_3.jpg</t>
+  </si>
+  <si>
+    <t>images/wallets/1641259664_4.jpg</t>
+  </si>
+  <si>
+    <t>images/wallets/712599567_2.jpg</t>
+  </si>
+  <si>
+    <t>images/wallets/712599567_3.jpg</t>
+  </si>
+  <si>
+    <t>images/wallets/712599567_4.jpg</t>
+  </si>
+  <si>
+    <t>images/belts/4497437028_2.jpg</t>
+  </si>
+  <si>
+    <t>images/belts/4497437028_3.jpg</t>
+  </si>
+  <si>
+    <t>images/belts/4497437028_4.jpg</t>
+  </si>
+  <si>
+    <t>images/belts/4497421494_2.jpeg</t>
+  </si>
+  <si>
+    <t>images/belts/4497421494_3.jpeg</t>
+  </si>
+  <si>
+    <t>images/belts/4497421494_4.jpeg</t>
+  </si>
+  <si>
+    <t>images/belts/4497421419_2.jpg</t>
+  </si>
+  <si>
+    <t>images/belts/4497421419_3.jpg</t>
+  </si>
+  <si>
+    <t>images/belts/4497421419_4.jpg</t>
+  </si>
+  <si>
+    <t>images/belts/4518376787_2.jpg</t>
+  </si>
+  <si>
+    <t>images/belts/4518376787_3.jpg</t>
+  </si>
+  <si>
+    <t>images/belts/4518376787_4.jpg</t>
+  </si>
+  <si>
+    <t>images/belts/4507840144_2.jpg</t>
+  </si>
+  <si>
+    <t>images/belts/4507840144_3.jpg</t>
+  </si>
+  <si>
+    <t>images/belts/4507840144_4.jpg</t>
+  </si>
+  <si>
+    <t>images/belts/4507832399_2.jpg</t>
+  </si>
+  <si>
+    <t>images/belts/4507832399_3.jpg</t>
+  </si>
+  <si>
+    <t>images/belts/4507832399_4.jpg</t>
+  </si>
+  <si>
+    <t>images/edc/1854958967_2.jpg</t>
+  </si>
+  <si>
+    <t>images/edc/1854958967_4.jpg</t>
+  </si>
+  <si>
+    <t>images/edc/1854958967_3.jpg</t>
+  </si>
+  <si>
+    <t>images/edc/1115911348_2.jpg</t>
+  </si>
+  <si>
+    <t>images/edc/1115911348_3.jpg</t>
+  </si>
+  <si>
+    <t>images/edc/1115911348_4.jpg</t>
+  </si>
+  <si>
+    <t>images/edc/4538303179_2.jpg</t>
+  </si>
+  <si>
+    <t>images/edc/4538303179_3.jpg</t>
+  </si>
+  <si>
+    <t>images/edc/4538303179_4.jpg</t>
+  </si>
+  <si>
+    <t>images/edc/1677683372_2.jpg</t>
+  </si>
+  <si>
+    <t>images/edc/1677683372_3.jpg</t>
+  </si>
+  <si>
+    <t>images/edc/1677683372_4.jpg</t>
+  </si>
+  <si>
+    <t>images/edc/4505762718_2.jpg</t>
+  </si>
+  <si>
+    <t>images/edc/4505762718_3.jpg</t>
+  </si>
+  <si>
+    <t>images/edc/4505762718_4.jpg</t>
+  </si>
+  <si>
+    <t>images/edc/4384063617_2.jpg</t>
+  </si>
+  <si>
+    <t>images/edc/4384063617_3.jpg</t>
+  </si>
+  <si>
+    <t>images/edc/4384063617_4.jpg</t>
+  </si>
+  <si>
+    <t>images/edc/4559330701_2.jpg</t>
+  </si>
+  <si>
+    <t>images/edc/4559330701_3.jpg</t>
+  </si>
+  <si>
+    <t>images/edc/4559330701_4.jpg</t>
+  </si>
+  <si>
+    <t>images/edc/4524136544_2.jpg</t>
+  </si>
+  <si>
+    <t>images/edc/4524136544_3.jpg</t>
+  </si>
+  <si>
+    <t>images/edc/4524136544_4.jpg</t>
+  </si>
+  <si>
+    <t>images/edc/1815374701_2.jpg</t>
+  </si>
+  <si>
+    <t>images/edc/1815374701_3.jpg</t>
+  </si>
+  <si>
+    <t>images/edc/1815374701_4.jpg</t>
+  </si>
+  <si>
+    <t>images/edc/4497871197_2.jpg</t>
+  </si>
+  <si>
+    <t>images/edc/4497871197_3.jpg</t>
+  </si>
+  <si>
+    <t>images/edc/4497871197_4.jpg</t>
+  </si>
+  <si>
+    <t>images/edc/4546239570_2.jpg</t>
+  </si>
+  <si>
+    <t>images/edc/4546239570_3.jpg</t>
+  </si>
+  <si>
+    <t>images/edc/4546239570_4.jpg</t>
+  </si>
+  <si>
+    <t>images/edc/1126874991_2.jpg</t>
+  </si>
+  <si>
+    <t>images/edc/1126874991_3.jpg</t>
+  </si>
+  <si>
+    <t>images/edc/1126874991_4.jpg</t>
+  </si>
+  <si>
+    <t>images/edc/4361026591_2.jpg</t>
+  </si>
+  <si>
+    <t>images/edc/4361026591_3.jpg</t>
+  </si>
+  <si>
+    <t>images/edc/4361026591_4.jpg</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -517,13 +751,26 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
+      <family val="2"/>
+      <charset val="204"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -539,7 +786,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -557,6 +804,15 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="2" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Гиперссылка" xfId="1" builtinId="8"/>
@@ -859,7 +1115,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:N30"/>
+  <dimension ref="A1:Q30"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -871,9 +1127,12 @@
     <col min="8" max="8" width="11.42578125" customWidth="1"/>
     <col min="9" max="9" width="9.140625" style="10"/>
     <col min="10" max="10" width="9.140625" style="8"/>
+    <col min="15" max="15" width="29.42578125" customWidth="1"/>
+    <col min="16" max="16" width="31.28515625" customWidth="1"/>
+    <col min="17" max="17" width="30.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:17" ht="15.75" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
         <v>38</v>
       </c>
@@ -916,8 +1175,17 @@
       <c r="N1" s="9" t="s">
         <v>151</v>
       </c>
-    </row>
-    <row r="2" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="O1" s="11" t="s">
+        <v>152</v>
+      </c>
+      <c r="P1" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="Q1" s="11" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -961,8 +1229,17 @@
       <c r="N2">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="O2" t="s">
+        <v>161</v>
+      </c>
+      <c r="P2" t="s">
+        <v>162</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
@@ -1006,8 +1283,17 @@
       <c r="N3">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="O3" t="s">
+        <v>158</v>
+      </c>
+      <c r="P3" t="s">
+        <v>159</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>0</v>
       </c>
@@ -1051,8 +1337,17 @@
       <c r="N4">
         <v>1</v>
       </c>
-    </row>
-    <row r="5" spans="1:14" ht="45" x14ac:dyDescent="0.25">
+      <c r="O4" t="s">
+        <v>155</v>
+      </c>
+      <c r="P4" t="s">
+        <v>156</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" ht="45" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>0</v>
       </c>
@@ -1096,8 +1391,17 @@
       <c r="N5">
         <v>1</v>
       </c>
-    </row>
-    <row r="6" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="O5" t="s">
+        <v>164</v>
+      </c>
+      <c r="P5" t="s">
+        <v>165</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>1</v>
       </c>
@@ -1141,8 +1445,17 @@
       <c r="N6">
         <v>1</v>
       </c>
-    </row>
-    <row r="7" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="O6" t="s">
+        <v>167</v>
+      </c>
+      <c r="P6" t="s">
+        <v>168</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>1</v>
       </c>
@@ -1186,8 +1499,17 @@
       <c r="N7">
         <v>1</v>
       </c>
-    </row>
-    <row r="8" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="O7" t="s">
+        <v>170</v>
+      </c>
+      <c r="P7" t="s">
+        <v>171</v>
+      </c>
+      <c r="Q7" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>2</v>
       </c>
@@ -1231,8 +1553,17 @@
       <c r="N8">
         <v>1</v>
       </c>
-    </row>
-    <row r="9" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="O8" t="s">
+        <v>173</v>
+      </c>
+      <c r="P8" t="s">
+        <v>174</v>
+      </c>
+      <c r="Q8" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>2</v>
       </c>
@@ -1276,8 +1607,17 @@
       <c r="N9">
         <v>1</v>
       </c>
-    </row>
-    <row r="10" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="O9" t="s">
+        <v>176</v>
+      </c>
+      <c r="P9" t="s">
+        <v>177</v>
+      </c>
+      <c r="Q9" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>2</v>
       </c>
@@ -1321,8 +1661,17 @@
       <c r="N10">
         <v>1</v>
       </c>
-    </row>
-    <row r="11" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="O10" t="s">
+        <v>179</v>
+      </c>
+      <c r="P10" t="s">
+        <v>180</v>
+      </c>
+      <c r="Q10" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="11" spans="1:17" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>2</v>
       </c>
@@ -1366,8 +1715,17 @@
       <c r="N11">
         <v>1</v>
       </c>
-    </row>
-    <row r="12" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="O11" t="s">
+        <v>182</v>
+      </c>
+      <c r="P11" t="s">
+        <v>183</v>
+      </c>
+      <c r="Q11" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="12" spans="1:17" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>2</v>
       </c>
@@ -1411,8 +1769,17 @@
       <c r="N12">
         <v>1</v>
       </c>
-    </row>
-    <row r="13" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="O12" t="s">
+        <v>185</v>
+      </c>
+      <c r="P12" t="s">
+        <v>186</v>
+      </c>
+      <c r="Q12" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="13" spans="1:17" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>2</v>
       </c>
@@ -1456,53 +1823,62 @@
       <c r="N13">
         <v>1</v>
       </c>
-    </row>
-    <row r="14" spans="1:14" ht="30" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
+      <c r="O13" t="s">
+        <v>188</v>
+      </c>
+      <c r="P13" t="s">
+        <v>189</v>
+      </c>
+      <c r="Q13" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="14" spans="1:17" s="14" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A14" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B14" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="C14" t="s">
+      <c r="C14" s="14" t="s">
         <v>82</v>
       </c>
-      <c r="D14" t="s">
+      <c r="D14" s="14" t="s">
         <v>27</v>
       </c>
-      <c r="E14" t="s">
+      <c r="E14" s="14" t="s">
         <v>58</v>
       </c>
-      <c r="F14" t="s">
+      <c r="F14" s="14" t="s">
         <v>101</v>
       </c>
-      <c r="G14" t="s">
+      <c r="G14" s="14" t="s">
         <v>107</v>
       </c>
-      <c r="H14" t="s">
+      <c r="H14" s="14" t="s">
         <v>44</v>
       </c>
-      <c r="I14" s="10">
+      <c r="I14" s="15">
         <f t="shared" si="0"/>
         <v>39.200000000000003</v>
       </c>
-      <c r="J14" s="8" t="s">
-        <v>110</v>
-      </c>
-      <c r="K14">
+      <c r="J14" s="16" t="s">
+        <v>110</v>
+      </c>
+      <c r="K14" s="14">
         <v>15</v>
       </c>
-      <c r="L14">
-        <v>20</v>
-      </c>
-      <c r="M14" s="10">
+      <c r="L14" s="14">
+        <v>20</v>
+      </c>
+      <c r="M14" s="15">
         <v>49</v>
       </c>
-      <c r="N14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="N14" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:17" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>3</v>
       </c>
@@ -1546,8 +1922,17 @@
       <c r="N15">
         <v>1</v>
       </c>
-    </row>
-    <row r="16" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="O15" t="s">
+        <v>191</v>
+      </c>
+      <c r="P15" t="s">
+        <v>193</v>
+      </c>
+      <c r="Q15" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="16" spans="1:17" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>3</v>
       </c>
@@ -1591,8 +1976,17 @@
       <c r="N16">
         <v>1</v>
       </c>
-    </row>
-    <row r="17" spans="1:14" ht="60" x14ac:dyDescent="0.25">
+      <c r="O16" t="s">
+        <v>194</v>
+      </c>
+      <c r="P16" t="s">
+        <v>195</v>
+      </c>
+      <c r="Q16" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="17" spans="1:17" ht="60" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>3</v>
       </c>
@@ -1636,8 +2030,17 @@
       <c r="N17">
         <v>1</v>
       </c>
-    </row>
-    <row r="18" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="O17" t="s">
+        <v>197</v>
+      </c>
+      <c r="P17" t="s">
+        <v>198</v>
+      </c>
+      <c r="Q17" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="18" spans="1:17" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>3</v>
       </c>
@@ -1681,53 +2084,62 @@
       <c r="N18">
         <v>1</v>
       </c>
-    </row>
-    <row r="19" spans="1:14" ht="60" x14ac:dyDescent="0.25">
-      <c r="A19" s="1" t="s">
+      <c r="O18" t="s">
+        <v>200</v>
+      </c>
+      <c r="P18" t="s">
+        <v>201</v>
+      </c>
+      <c r="Q18" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="19" spans="1:17" s="14" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+      <c r="A19" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="B19" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="C19" t="s">
+      <c r="C19" s="14" t="s">
         <v>87</v>
       </c>
-      <c r="D19" t="s">
+      <c r="D19" s="14" t="s">
         <v>37</v>
       </c>
-      <c r="E19" t="s">
+      <c r="E19" s="14" t="s">
         <v>63</v>
       </c>
-      <c r="F19" t="s">
+      <c r="F19" s="14" t="s">
         <v>106</v>
       </c>
-      <c r="G19" t="s">
+      <c r="G19" s="14" t="s">
         <v>107</v>
       </c>
-      <c r="H19" t="s">
+      <c r="H19" s="14" t="s">
         <v>44</v>
       </c>
-      <c r="I19" s="10">
+      <c r="I19" s="15">
         <f t="shared" si="0"/>
         <v>55.2</v>
       </c>
-      <c r="J19" s="8" t="s">
-        <v>110</v>
-      </c>
-      <c r="K19">
+      <c r="J19" s="16" t="s">
+        <v>110</v>
+      </c>
+      <c r="K19" s="14">
         <v>15</v>
       </c>
-      <c r="L19">
-        <v>20</v>
-      </c>
-      <c r="M19" s="10">
+      <c r="L19" s="14">
+        <v>20</v>
+      </c>
+      <c r="M19" s="15">
         <v>69</v>
       </c>
-      <c r="N19">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="20" spans="1:14" ht="45" x14ac:dyDescent="0.25">
+      <c r="N19" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:17" ht="45" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>3</v>
       </c>
@@ -1771,8 +2183,17 @@
       <c r="N20">
         <v>1</v>
       </c>
-    </row>
-    <row r="21" spans="1:14" ht="45" x14ac:dyDescent="0.25">
+      <c r="O20" t="s">
+        <v>203</v>
+      </c>
+      <c r="P20" t="s">
+        <v>204</v>
+      </c>
+      <c r="Q20" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="21" spans="1:17" ht="45" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>3</v>
       </c>
@@ -1816,8 +2237,17 @@
       <c r="N21">
         <v>1</v>
       </c>
-    </row>
-    <row r="22" spans="1:14" ht="45" x14ac:dyDescent="0.25">
+      <c r="O21" t="s">
+        <v>206</v>
+      </c>
+      <c r="P21" t="s">
+        <v>207</v>
+      </c>
+      <c r="Q21" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="22" spans="1:17" ht="45" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>3</v>
       </c>
@@ -1861,8 +2291,17 @@
       <c r="N22">
         <v>1</v>
       </c>
-    </row>
-    <row r="23" spans="1:14" ht="45" x14ac:dyDescent="0.25">
+      <c r="O22" t="s">
+        <v>209</v>
+      </c>
+      <c r="P22" t="s">
+        <v>210</v>
+      </c>
+      <c r="Q22" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="23" spans="1:17" ht="45" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>3</v>
       </c>
@@ -1906,8 +2345,17 @@
       <c r="N23">
         <v>1</v>
       </c>
-    </row>
-    <row r="24" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="O23" t="s">
+        <v>212</v>
+      </c>
+      <c r="P23" t="s">
+        <v>213</v>
+      </c>
+      <c r="Q23" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="24" spans="1:17" ht="30" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>3</v>
       </c>
@@ -1951,53 +2399,62 @@
       <c r="N24">
         <v>1</v>
       </c>
-    </row>
-    <row r="25" spans="1:14" ht="45" x14ac:dyDescent="0.25">
-      <c r="A25" s="1" t="s">
+      <c r="O24" t="s">
+        <v>215</v>
+      </c>
+      <c r="P24" t="s">
+        <v>216</v>
+      </c>
+      <c r="Q24" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="25" spans="1:17" s="14" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+      <c r="A25" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="B25" s="2" t="s">
+      <c r="B25" s="13" t="s">
         <v>127</v>
       </c>
-      <c r="C25" t="s">
+      <c r="C25" s="14" t="s">
         <v>86</v>
       </c>
-      <c r="D25" s="6" t="s">
+      <c r="D25" s="17" t="s">
         <v>128</v>
       </c>
-      <c r="E25" t="s">
+      <c r="E25" s="14" t="s">
         <v>129</v>
       </c>
-      <c r="F25" t="s">
+      <c r="F25" s="14" t="s">
         <v>121</v>
       </c>
-      <c r="G25" t="s">
+      <c r="G25" s="14" t="s">
         <v>107</v>
       </c>
-      <c r="H25" t="s">
+      <c r="H25" s="14" t="s">
         <v>44</v>
       </c>
-      <c r="I25" s="10">
+      <c r="I25" s="15">
         <f t="shared" si="0"/>
         <v>55.2</v>
       </c>
-      <c r="J25" s="8" t="s">
-        <v>110</v>
-      </c>
-      <c r="K25">
+      <c r="J25" s="16" t="s">
+        <v>110</v>
+      </c>
+      <c r="K25" s="14">
         <v>15</v>
       </c>
-      <c r="L25">
-        <v>20</v>
-      </c>
-      <c r="M25" s="10">
+      <c r="L25" s="14">
+        <v>20</v>
+      </c>
+      <c r="M25" s="15">
         <v>69</v>
       </c>
-      <c r="N25">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="26" spans="1:14" ht="45" x14ac:dyDescent="0.25">
+      <c r="N25" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:17" ht="45" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>0</v>
       </c>
@@ -2042,7 +2499,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:14" ht="45" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:17" ht="45" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>3</v>
       </c>
@@ -2086,8 +2543,17 @@
       <c r="N27">
         <v>1</v>
       </c>
-    </row>
-    <row r="28" spans="1:14" ht="45" x14ac:dyDescent="0.25">
+      <c r="O27" t="s">
+        <v>218</v>
+      </c>
+      <c r="P27" t="s">
+        <v>219</v>
+      </c>
+      <c r="Q27" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="28" spans="1:17" ht="45" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>3</v>
       </c>
@@ -2131,8 +2597,17 @@
       <c r="N28">
         <v>1</v>
       </c>
-    </row>
-    <row r="29" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="O28" t="s">
+        <v>221</v>
+      </c>
+      <c r="P28" t="s">
+        <v>222</v>
+      </c>
+      <c r="Q28" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="29" spans="1:17" ht="30" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>3</v>
       </c>
@@ -2173,8 +2648,17 @@
       <c r="N29">
         <v>1</v>
       </c>
-    </row>
-    <row r="30" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="O29" t="s">
+        <v>227</v>
+      </c>
+      <c r="P29" t="s">
+        <v>228</v>
+      </c>
+      <c r="Q29" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="30" spans="1:17" ht="30" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>3</v>
       </c>
@@ -2217,6 +2701,15 @@
       </c>
       <c r="N30">
         <v>1</v>
+      </c>
+      <c r="O30" t="s">
+        <v>224</v>
+      </c>
+      <c r="P30" t="s">
+        <v>225</v>
+      </c>
+      <c r="Q30" t="s">
+        <v>226</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add three new leather EDC products
</commit_message>
<xml_diff>
--- a/goods(4).xlsx
+++ b/goods(4).xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="361" uniqueCount="230">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="397" uniqueCount="245">
   <si>
     <t>Bags</t>
   </si>
@@ -705,6 +705,51 @@
   </si>
   <si>
     <t>images/edc/4361026591_4.jpg</t>
+  </si>
+  <si>
+    <t>https://www.etsy.com/listing/4598044441</t>
+  </si>
+  <si>
+    <t>images/edc/4598044441.jpg</t>
+  </si>
+  <si>
+    <t>images/edc/4598044441_2.jpg</t>
+  </si>
+  <si>
+    <t>images/edc/4598044441_3.jpg</t>
+  </si>
+  <si>
+    <t>images/edc/4598044441_4.jpg</t>
+  </si>
+  <si>
+    <t>https://www.etsy.com/listing/4599487751</t>
+  </si>
+  <si>
+    <t>images/edc/4599487751.jpg</t>
+  </si>
+  <si>
+    <t>images/edc/4599487751_2.jpg</t>
+  </si>
+  <si>
+    <t>images/edc/4599487751_3.jpg</t>
+  </si>
+  <si>
+    <t>images/edc/4599487751_4.jpg</t>
+  </si>
+  <si>
+    <t>https://www.etsy.com/listing/4601714691</t>
+  </si>
+  <si>
+    <t>images/edc/4601714691.jpg</t>
+  </si>
+  <si>
+    <t>images/edc/4601714691_2.jpg</t>
+  </si>
+  <si>
+    <t>images/edc/4601714691_3.jpg</t>
+  </si>
+  <si>
+    <t>images/edc/4601714691_4.jpg</t>
   </si>
 </sst>
 </file>
@@ -1115,7 +1160,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Q30"/>
+  <dimension ref="A1:Q33"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -2712,6 +2757,168 @@
         <v>226</v>
       </c>
     </row>
+    <row r="31" spans="1:17" ht="30" x14ac:dyDescent="0.25">
+      <c r="A31" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C31" t="s">
+        <v>84</v>
+      </c>
+      <c r="D31" s="6" t="s">
+        <v>230</v>
+      </c>
+      <c r="E31" t="s">
+        <v>231</v>
+      </c>
+      <c r="F31" t="s">
+        <v>147</v>
+      </c>
+      <c r="G31" t="s">
+        <v>43</v>
+      </c>
+      <c r="H31" t="s">
+        <v>44</v>
+      </c>
+      <c r="I31" s="10">
+        <f t="shared" ref="I31" si="1">M31-PRODUCT(M31,L31)/100</f>
+        <v>55.2</v>
+      </c>
+      <c r="J31" s="8" t="s">
+        <v>110</v>
+      </c>
+      <c r="K31">
+        <v>15</v>
+      </c>
+      <c r="L31">
+        <v>20</v>
+      </c>
+      <c r="M31" s="10">
+        <v>69</v>
+      </c>
+      <c r="N31">
+        <v>1</v>
+      </c>
+      <c r="O31" t="s">
+        <v>232</v>
+      </c>
+      <c r="P31" t="s">
+        <v>233</v>
+      </c>
+      <c r="Q31" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="32" spans="1:17" ht="30" x14ac:dyDescent="0.25">
+      <c r="A32" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C32" t="s">
+        <v>84</v>
+      </c>
+      <c r="D32" s="6" t="s">
+        <v>235</v>
+      </c>
+      <c r="E32" t="s">
+        <v>236</v>
+      </c>
+      <c r="F32" t="s">
+        <v>147</v>
+      </c>
+      <c r="G32" t="s">
+        <v>43</v>
+      </c>
+      <c r="H32" t="s">
+        <v>44</v>
+      </c>
+      <c r="I32" s="10">
+        <f t="shared" ref="I32" si="2">M32-PRODUCT(M32,L32)/100</f>
+        <v>55.2</v>
+      </c>
+      <c r="J32" s="8" t="s">
+        <v>110</v>
+      </c>
+      <c r="K32">
+        <v>15</v>
+      </c>
+      <c r="L32">
+        <v>20</v>
+      </c>
+      <c r="M32" s="10">
+        <v>69</v>
+      </c>
+      <c r="N32">
+        <v>1</v>
+      </c>
+      <c r="O32" t="s">
+        <v>237</v>
+      </c>
+      <c r="P32" t="s">
+        <v>238</v>
+      </c>
+      <c r="Q32" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="33" spans="1:17" ht="30" x14ac:dyDescent="0.25">
+      <c r="A33" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C33" t="s">
+        <v>84</v>
+      </c>
+      <c r="D33" s="6" t="s">
+        <v>240</v>
+      </c>
+      <c r="E33" t="s">
+        <v>241</v>
+      </c>
+      <c r="F33" t="s">
+        <v>147</v>
+      </c>
+      <c r="G33" t="s">
+        <v>43</v>
+      </c>
+      <c r="H33" t="s">
+        <v>44</v>
+      </c>
+      <c r="I33" s="10">
+        <f t="shared" ref="I33" si="3">M33-PRODUCT(M33,L33)/100</f>
+        <v>55.2</v>
+      </c>
+      <c r="J33" s="8" t="s">
+        <v>110</v>
+      </c>
+      <c r="K33">
+        <v>15</v>
+      </c>
+      <c r="L33">
+        <v>20</v>
+      </c>
+      <c r="M33" s="10">
+        <v>69</v>
+      </c>
+      <c r="N33">
+        <v>1</v>
+      </c>
+      <c r="O33" t="s">
+        <v>242</v>
+      </c>
+      <c r="P33" t="s">
+        <v>243</v>
+      </c>
+      <c r="Q33" t="s">
+        <v>244</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="D2" r:id="rId1"/>
@@ -2723,9 +2930,12 @@
     <hyperlink ref="D28" r:id="rId7"/>
     <hyperlink ref="D29" r:id="rId8"/>
     <hyperlink ref="D30" r:id="rId9"/>
+    <hyperlink ref="D31" r:id="rId10"/>
+    <hyperlink ref="D32" r:id="rId11"/>
+    <hyperlink ref="D33" r:id="rId12"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId10"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId13"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Remove sold product and update product details
</commit_message>
<xml_diff>
--- a/goods(4).xlsx
+++ b/goods(4).xlsx
@@ -1263,7 +1263,7 @@
         <v>110</v>
       </c>
       <c r="K2">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="L2">
         <v>20</v>
@@ -1317,7 +1317,7 @@
         <v>110</v>
       </c>
       <c r="K3">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="L3">
         <v>20</v>
@@ -2499,48 +2499,48 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:17" ht="45" x14ac:dyDescent="0.25">
-      <c r="A26" s="1" t="s">
+    <row r="26" spans="1:17" s="14" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+      <c r="A26" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B26" s="2" t="s">
+      <c r="B26" s="13" t="s">
         <v>130</v>
       </c>
-      <c r="C26" t="s">
+      <c r="C26" s="14" t="s">
         <v>131</v>
       </c>
-      <c r="D26" s="6" t="s">
+      <c r="D26" s="17" t="s">
         <v>132</v>
       </c>
-      <c r="E26" t="s">
+      <c r="E26" s="14" t="s">
         <v>133</v>
       </c>
-      <c r="F26" t="s">
+      <c r="F26" s="14" t="s">
         <v>134</v>
       </c>
-      <c r="G26" t="s">
-        <v>43</v>
-      </c>
-      <c r="H26" t="s">
+      <c r="G26" s="14" t="s">
+        <v>107</v>
+      </c>
+      <c r="H26" s="14" t="s">
         <v>44</v>
       </c>
-      <c r="I26" s="10">
+      <c r="I26" s="15">
         <f t="shared" si="0"/>
         <v>69.599999999999994</v>
       </c>
-      <c r="J26" s="8" t="s">
-        <v>110</v>
-      </c>
-      <c r="K26">
+      <c r="J26" s="16" t="s">
+        <v>110</v>
+      </c>
+      <c r="K26" s="14">
         <v>15</v>
       </c>
-      <c r="L26">
-        <v>20</v>
-      </c>
-      <c r="M26" s="10">
+      <c r="L26" s="14">
+        <v>20</v>
+      </c>
+      <c r="M26" s="15">
         <v>87</v>
       </c>
-      <c r="N26">
+      <c r="N26" s="14">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add  leather belt pouch product pages
</commit_message>
<xml_diff>
--- a/goods(4).xlsx
+++ b/goods(4).xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="397" uniqueCount="245">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="400" uniqueCount="248">
   <si>
     <t>Bags</t>
   </si>
@@ -750,6 +750,15 @@
   </si>
   <si>
     <t>images/edc/4601714691_4.jpg</t>
+  </si>
+  <si>
+    <t>images/edc/4590678904_2.jpg</t>
+  </si>
+  <si>
+    <t>images/edc/4590678904_3.jpg</t>
+  </si>
+  <si>
+    <t>images/edc/4590678904_4.jpg</t>
   </si>
 </sst>
 </file>
@@ -804,7 +813,7 @@
       <charset val="204"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -814,6 +823,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="6" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -831,7 +846,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -858,6 +873,14 @@
     <xf numFmtId="2" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="1" applyFill="1"/>
+    <xf numFmtId="2" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="49" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Гиперссылка" xfId="1" builtinId="8"/>
@@ -2454,49 +2477,58 @@
         <v>217</v>
       </c>
     </row>
-    <row r="25" spans="1:17" s="14" customFormat="1" ht="45" x14ac:dyDescent="0.25">
-      <c r="A25" s="12" t="s">
+    <row r="25" spans="1:17" s="20" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+      <c r="A25" s="18" t="s">
         <v>3</v>
       </c>
-      <c r="B25" s="13" t="s">
+      <c r="B25" s="19" t="s">
         <v>127</v>
       </c>
-      <c r="C25" s="14" t="s">
+      <c r="C25" s="20" t="s">
         <v>86</v>
       </c>
-      <c r="D25" s="17" t="s">
+      <c r="D25" s="21" t="s">
         <v>128</v>
       </c>
-      <c r="E25" s="14" t="s">
+      <c r="E25" s="20" t="s">
         <v>129</v>
       </c>
-      <c r="F25" s="14" t="s">
+      <c r="F25" s="20" t="s">
         <v>121</v>
       </c>
-      <c r="G25" s="14" t="s">
-        <v>107</v>
-      </c>
-      <c r="H25" s="14" t="s">
+      <c r="G25" s="20" t="s">
+        <v>43</v>
+      </c>
+      <c r="H25" s="20" t="s">
         <v>44</v>
       </c>
-      <c r="I25" s="15">
+      <c r="I25" s="22">
         <f t="shared" si="0"/>
         <v>55.2</v>
       </c>
-      <c r="J25" s="16" t="s">
-        <v>110</v>
-      </c>
-      <c r="K25" s="14">
+      <c r="J25" s="23" t="s">
+        <v>110</v>
+      </c>
+      <c r="K25" s="20">
         <v>15</v>
       </c>
-      <c r="L25" s="14">
-        <v>20</v>
-      </c>
-      <c r="M25" s="15">
+      <c r="L25" s="20">
+        <v>20</v>
+      </c>
+      <c r="M25" s="22">
         <v>69</v>
       </c>
-      <c r="N25" s="14">
-        <v>1</v>
+      <c r="N25" s="20">
+        <v>1</v>
+      </c>
+      <c r="O25" s="20" t="s">
+        <v>245</v>
+      </c>
+      <c r="P25" s="20" t="s">
+        <v>246</v>
+      </c>
+      <c r="Q25" s="20" t="s">
+        <v>247</v>
       </c>
     </row>
     <row r="26" spans="1:17" s="14" customFormat="1" ht="45" x14ac:dyDescent="0.25">

</xml_diff>